<commit_message>
feat: verify conditional and lookup formula families
</commit_message>
<xml_diff>
--- a/src-tauri/tests/fixtures/workbook/formula-function-matrix.xlsx
+++ b/src-tauri/tests/fixtures/workbook/formula-function-matrix.xlsx
@@ -8,13 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="Formula Matrix" sheetId="1" r:id="rId1"/>
+    <sheet name="Lookup Data" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
   <si>
     <t>Value</t>
   </si>
@@ -86,6 +87,81 @@
   </si>
   <si>
     <t>unknown_function</t>
+  </si>
+  <si>
+    <t>conditional_sumif</t>
+  </si>
+  <si>
+    <t>conditional_countif</t>
+  </si>
+  <si>
+    <t>conditional_averageif</t>
+  </si>
+  <si>
+    <t>conditional_wildcard</t>
+  </si>
+  <si>
+    <t>lookup_vlookup_exact</t>
+  </si>
+  <si>
+    <t>lookup_vlookup_approximate</t>
+  </si>
+  <si>
+    <t>lookup_hlookup_exact</t>
+  </si>
+  <si>
+    <t>lookup_index</t>
+  </si>
+  <si>
+    <t>lookup_match_exact</t>
+  </si>
+  <si>
+    <t>lookup_match_approximate</t>
+  </si>
+  <si>
+    <t>lookup_text_result</t>
+  </si>
+  <si>
+    <t>lookup_not_found</t>
+  </si>
+  <si>
+    <t>lookup_error_recovery</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Starter</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Basic</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Pro</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>400</t>
+  </si>
+  <si>
+    <t>Enterprise</t>
+  </si>
+  <si>
+    <t>E</t>
   </si>
 </sst>
 </file>
@@ -426,7 +502,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="16.7109375" customWidth="1"/>
@@ -625,6 +701,233 @@
         <v>#NAME?</v>
       </c>
     </row>
+    <row r="20" spans="4:5">
+      <c r="D20" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20">
+        <f>SUMIF(A2:A4,"&gt;15")</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="4:5">
+      <c r="D21" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21">
+        <f>COUNTIF(A2:A4,"&gt;=20")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="4:5">
+      <c r="D22" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22">
+        <f>AVERAGEIF(A2:A4,"&gt;10")</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="4:5">
+      <c r="D23" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23">
+        <f>COUNTIF('Lookup Data'!A2:A6,"?")</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="4:5">
+      <c r="D24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24">
+        <f>VLOOKUP("B",'Lookup Data'!A2:B6,2,FALSE)</f>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="25" spans="4:5">
+      <c r="D25" t="s">
+        <v>29</v>
+      </c>
+      <c r="E25" t="str">
+        <f>VLOOKUP(25,'Lookup Data'!E2:F5,2,TRUE)</f>
+        <v>Pro</v>
+      </c>
+    </row>
+    <row r="26" spans="4:5">
+      <c r="D26" t="s">
+        <v>30</v>
+      </c>
+      <c r="E26">
+        <f>HLOOKUP("C",'Lookup Data'!A8:D9,2,FALSE)</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="27" spans="4:5">
+      <c r="D27" t="s">
+        <v>31</v>
+      </c>
+      <c r="E27">
+        <f>INDEX('Lookup Data'!B2:B6,3)</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="28" spans="4:5">
+      <c r="D28" t="s">
+        <v>32</v>
+      </c>
+      <c r="E28">
+        <f>MATCH("C",'Lookup Data'!A2:A6,0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="4:5">
+      <c r="D29" t="s">
+        <v>33</v>
+      </c>
+      <c r="E29">
+        <f>MATCH(25,'Lookup Data'!E2:E5,1)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="4:5">
+      <c r="D30" t="s">
+        <v>34</v>
+      </c>
+      <c r="E30">
+        <f>VLOOKUP("D",'Lookup Data'!A2:B6,2,FALSE)</f>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="31" spans="4:5">
+      <c r="D31" t="s">
+        <v>35</v>
+      </c>
+      <c r="E31" t="e">
+        <f>VLOOKUP("Z",'Lookup Data'!A2:B6,2,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="32" spans="4:5">
+      <c r="D32" t="s">
+        <v>36</v>
+      </c>
+      <c r="E32" t="str">
+        <f>IFERROR(E31,"missing")</f>
+        <v>missing</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2">
+        <v>100</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3">
+        <v>200</v>
+      </c>
+      <c r="E3">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4">
+        <v>300</v>
+      </c>
+      <c r="E4">
+        <v>20</v>
+      </c>
+      <c r="F4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5">
+        <v>30</v>
+      </c>
+      <c r="F5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9">
+        <v>100</v>
+      </c>
+      <c r="B9">
+        <v>200</v>
+      </c>
+      <c r="C9">
+        <v>300</v>
+      </c>
+      <c r="D9">
+        <v>400</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add verified XMATCH calculation
</commit_message>
<xml_diff>
--- a/src-tauri/tests/fixtures/workbook/formula-function-matrix.xlsx
+++ b/src-tauri/tests/fixtures/workbook/formula-function-matrix.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="85">
   <si>
     <t>Value</t>
   </si>
@@ -232,6 +232,30 @@
   </si>
   <si>
     <t>volatile_clock_relation</t>
+  </si>
+  <si>
+    <t>xmatch_exact</t>
+  </si>
+  <si>
+    <t>xmatch_reverse_search</t>
+  </si>
+  <si>
+    <t>xmatch_wildcard</t>
+  </si>
+  <si>
+    <t>xmatch_next_smaller</t>
+  </si>
+  <si>
+    <t>xmatch_next_larger</t>
+  </si>
+  <si>
+    <t>xmatch_row_vector</t>
+  </si>
+  <si>
+    <t>xmatch_not_found</t>
+  </si>
+  <si>
+    <t>xmatch_error_recovery</t>
   </si>
   <si>
     <t>Code</t>
@@ -608,7 +632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="16.7109375" customWidth="1"/>
@@ -1159,6 +1183,78 @@
       <c r="E57" t="b">
         <f>AND(TODAY()&lt;=NOW(),NOW()&lt;TODAY()+1)</f>
         <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="4:5">
+      <c r="D58" t="s">
+        <v>65</v>
+      </c>
+      <c r="E58">
+        <f>_xlfn.XMATCH("C",'Lookup Data'!A2:A6)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="59" spans="4:5">
+      <c r="D59" t="s">
+        <v>66</v>
+      </c>
+      <c r="E59">
+        <f>_xlfn.XMATCH("East",C2:C4,0,-1)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="60" spans="4:5">
+      <c r="D60" t="s">
+        <v>67</v>
+      </c>
+      <c r="E60">
+        <f>_xlfn.XMATCH("C*",'Lookup Data'!A2:A6,2)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="61" spans="4:5">
+      <c r="D61" t="s">
+        <v>68</v>
+      </c>
+      <c r="E61">
+        <f>_xlfn.XMATCH(25,'Lookup Data'!E2:E5,-1)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="62" spans="4:5">
+      <c r="D62" t="s">
+        <v>69</v>
+      </c>
+      <c r="E62">
+        <f>_xlfn.XMATCH(25,'Lookup Data'!E2:E5,1)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63" spans="4:5">
+      <c r="D63" t="s">
+        <v>70</v>
+      </c>
+      <c r="E63">
+        <f>_xlfn.XMATCH("C",'Lookup Data'!A8:D8)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="64" spans="4:5">
+      <c r="D64" t="s">
+        <v>71</v>
+      </c>
+      <c r="E64" t="e">
+        <f>_xlfn.XMATCH("Z",'Lookup Data'!A2:A6)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="65" spans="4:5">
+      <c r="D65" t="s">
+        <v>72</v>
+      </c>
+      <c r="E65" t="str">
+        <f>IFERROR(E64,"recovered")</f>
+        <v>recovered</v>
       </c>
     </row>
   </sheetData>
@@ -1173,15 +1269,15 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="B1" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="B2">
         <v>100</v>
@@ -1190,12 +1286,12 @@
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="B3">
         <v>200</v>
@@ -1204,12 +1300,12 @@
         <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="B4">
         <v>300</v>
@@ -1218,26 +1314,26 @@
         <v>20</v>
       </c>
       <c r="F4" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="B5" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="E5">
         <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="B6">
         <v>500</v>
@@ -1245,16 +1341,16 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="C8" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="D8" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:6">

</xml_diff>